<commit_message>
[wip] attack pipline 6
</commit_message>
<xml_diff>
--- a/table_config/_tables/Battle/#EffectData-效果-01.xlsx
+++ b/table_config/_tables/Battle/#EffectData-效果-01.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23540" windowHeight="14150"/>
+    <workbookView windowWidth="27945" windowHeight="12375"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>##var</t>
   </si>
@@ -40,6 +40,9 @@
     <t>##别称</t>
   </si>
   <si>
+    <t>order</t>
+  </si>
+  <si>
     <t>luaScript</t>
   </si>
   <si>
@@ -65,6 +68,9 @@
   </si>
   <si>
     <t>唯一id</t>
+  </si>
+  <si>
+    <t>执行优先级</t>
   </si>
   <si>
     <t>lua脚本</t>
@@ -1020,15 +1026,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="5"/>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="5"/>
   <cols>
-    <col min="2" max="2" width="17.3636363636364" style="1"/>
-    <col min="3" max="4" width="16.2727272727273" style="2"/>
-    <col min="5" max="5" width="30.4545454545455" customWidth="1"/>
+    <col min="2" max="2" width="17.3666666666667" style="1"/>
+    <col min="3" max="3" width="16.275" style="2"/>
+    <col min="4" max="4" width="10.875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="16.275" style="2"/>
+    <col min="6" max="6" width="30.4583333333333" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1041,77 +1049,92 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3"/>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="3"/>
+      <c r="F2" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:10">
       <c r="A3" t="s">
         <v>0</v>
       </c>
-      <c r="E3" t="s">
-        <v>9</v>
+      <c r="F3" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:10">
       <c r="B5" s="1">
         <v>1001000001</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:10">
       <c r="B6" s="1">
         <v>1001000002</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="D6" s="2">
+        <v>2</v>
+      </c>
+      <c r="F6" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="E1:I1"/>
-    <mergeCell ref="E2:I2"/>
+    <mergeCell ref="F1:J1"/>
+    <mergeCell ref="F2:J2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -1123,7 +1146,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -1135,7 +1158,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
[wip] attack pipline 9
</commit_message>
<xml_diff>
--- a/table_config/_tables/Battle/#EffectData-效果-01.xlsx
+++ b/table_config/_tables/Battle/#EffectData-效果-01.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
   <si>
     <t>##var</t>
   </si>
@@ -40,15 +40,12 @@
     <t>##别称</t>
   </si>
   <si>
-    <t>order</t>
+    <t>tag</t>
   </si>
   <si>
     <t>luaScript</t>
   </si>
   <si>
-    <t>parameters</t>
-  </si>
-  <si>
     <t>##type</t>
   </si>
   <si>
@@ -58,34 +55,22 @@
     <t>string</t>
   </si>
   <si>
-    <t>Battle.EffectParamBase</t>
-  </si>
-  <si>
-    <t>$type</t>
-  </si>
-  <si>
     <t>##</t>
   </si>
   <si>
     <t>唯一id</t>
   </si>
   <si>
-    <t>执行优先级</t>
-  </si>
-  <si>
     <t>lua脚本</t>
   </si>
   <si>
-    <t>攻击</t>
-  </si>
-  <si>
-    <t>Battle.EffectAttack</t>
-  </si>
-  <si>
-    <t>受伤</t>
-  </si>
-  <si>
-    <t>Battle.EffectHurt</t>
+    <t>免疫所有伤害</t>
+  </si>
+  <si>
+    <t>battle</t>
+  </si>
+  <si>
+    <t>on_deal_damage_check_tag</t>
   </si>
 </sst>
 </file>
@@ -702,7 +687,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -711,9 +696,6 @@
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1026,17 +1008,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="5"/>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="4" outlineLevelCol="4"/>
   <cols>
     <col min="2" max="2" width="17.3666666666667" style="1"/>
     <col min="3" max="3" width="16.275" style="2"/>
-    <col min="4" max="4" width="10.875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="16.275" style="2"/>
-    <col min="6" max="6" width="30.4583333333333" customWidth="1"/>
+    <col min="4" max="4" width="7.375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="34.875" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1052,90 +1033,52 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-    </row>
-    <row r="2" spans="1:10">
-      <c r="A2" t="s">
+      <c r="B2" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>7</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
+        <v>7</v>
+      </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>0</v>
       </c>
-      <c r="F3" t="s">
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:5">
       <c r="B5" s="1">
         <v>1001000001</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="2">
-        <v>1</v>
-      </c>
-      <c r="F5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="B6" s="1">
-        <v>1001000002</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="2">
-        <v>2</v>
-      </c>
-      <c r="F6" t="s">
-        <v>18</v>
+        <v>11</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="F1:J1"/>
-    <mergeCell ref="F2:J2"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>

</xml_diff>